<commit_message>
Actualizacion del Documento de Especificacion Funcional
</commit_message>
<xml_diff>
--- a/docs/reportes_ejemplo/Reporte_BI_AromaGrano_7-5-2026.xlsx
+++ b/docs/reportes_ejemplo/Reporte_BI_AromaGrano_7-5-2026.xlsx
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:G3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -432,7 +432,7 @@
         <v>7/5/2026</v>
       </c>
       <c r="C2" t="str">
-        <v>7:30:29 AM</v>
+        <v>9:19:01 PM</v>
       </c>
       <c r="D2" t="str">
         <v>Mesa 1</v>
@@ -444,7 +444,7 @@
         <v>cerrado</v>
       </c>
       <c r="G2" t="str">
-        <v>30.00</v>
+        <v>34.01</v>
       </c>
     </row>
     <row r="3">
@@ -455,7 +455,7 @@
         <v>7/5/2026</v>
       </c>
       <c r="C3" t="str">
-        <v>7:55:25 AM</v>
+        <v>9:19:53 PM</v>
       </c>
       <c r="D3" t="str">
         <v>Mesa 1</v>
@@ -467,42 +467,19 @@
         <v>cerrado</v>
       </c>
       <c r="G3" t="str">
-        <v>3.40</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4">
-        <v>4</v>
-      </c>
-      <c r="B4" t="str">
-        <v>7/5/2026</v>
-      </c>
-      <c r="C4" t="str">
-        <v>8:21:20 AM</v>
-      </c>
-      <c r="D4" t="str">
-        <v>Mesa 1</v>
-      </c>
-      <c r="E4" t="str">
-        <v>Ana Maria</v>
-      </c>
-      <c r="F4" t="str">
-        <v>cerrado</v>
-      </c>
-      <c r="G4" t="str">
-        <v>8.00</v>
+        <v>10.00</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G3"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:K6"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -544,51 +521,51 @@
         <v>1</v>
       </c>
       <c r="B2" t="str">
-        <v>Cheesecake</v>
+        <v>Latte</v>
       </c>
       <c r="C2">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="D2" t="str">
-        <v>5.00</v>
+        <v>4.00</v>
       </c>
       <c r="E2" t="str">
-        <v>5.00</v>
+        <v>3.40</v>
       </c>
       <c r="F2" t="str">
-        <v>No</v>
+        <v>Sí</v>
       </c>
       <c r="G2">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="H2" t="str">
-        <v>0.00</v>
+        <v>0.60</v>
       </c>
       <c r="I2" t="str">
-        <v>30.00</v>
+        <v>3.40</v>
       </c>
       <c r="J2" t="str">
-        <v>13.20</v>
+        <v>1.50</v>
       </c>
       <c r="K2" t="str">
-        <v>16.80</v>
+        <v>1.90</v>
       </c>
     </row>
     <row r="3">
       <c r="A3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B3" t="str">
-        <v>Latte</v>
+        <v>Cappuccino</v>
       </c>
       <c r="C3">
         <v>1</v>
       </c>
       <c r="D3" t="str">
-        <v>4.00</v>
+        <v>3.50</v>
       </c>
       <c r="E3" t="str">
-        <v>3.40</v>
+        <v>2.98</v>
       </c>
       <c r="F3" t="str">
         <v>Sí</v>
@@ -597,56 +574,126 @@
         <v>15</v>
       </c>
       <c r="H3" t="str">
-        <v>0.60</v>
+        <v>0.52</v>
       </c>
       <c r="I3" t="str">
-        <v>3.40</v>
+        <v>2.98</v>
       </c>
       <c r="J3" t="str">
-        <v>1.50</v>
+        <v>1.20</v>
       </c>
       <c r="K3" t="str">
-        <v>1.90</v>
+        <v>1.78</v>
       </c>
     </row>
     <row r="4">
       <c r="A4">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="B4" t="str">
-        <v>Latte</v>
+        <v>Espresso</v>
       </c>
       <c r="C4">
+        <v>1</v>
+      </c>
+      <c r="D4" t="str">
+        <v>2.50</v>
+      </c>
+      <c r="E4" t="str">
+        <v>2.13</v>
+      </c>
+      <c r="F4" t="str">
+        <v>Sí</v>
+      </c>
+      <c r="G4">
+        <v>15</v>
+      </c>
+      <c r="H4" t="str">
+        <v>0.38</v>
+      </c>
+      <c r="I4" t="str">
+        <v>2.13</v>
+      </c>
+      <c r="J4" t="str">
+        <v>0.80</v>
+      </c>
+      <c r="K4" t="str">
+        <v>1.33</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5">
+        <v>1</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Cheesecake</v>
+      </c>
+      <c r="C5">
+        <v>6</v>
+      </c>
+      <c r="D5" t="str">
+        <v>5.00</v>
+      </c>
+      <c r="E5" t="str">
+        <v>4.25</v>
+      </c>
+      <c r="F5" t="str">
+        <v>Sí</v>
+      </c>
+      <c r="G5">
+        <v>15</v>
+      </c>
+      <c r="H5" t="str">
+        <v>0.75</v>
+      </c>
+      <c r="I5" t="str">
+        <v>25.50</v>
+      </c>
+      <c r="J5" t="str">
+        <v>13.20</v>
+      </c>
+      <c r="K5" t="str">
+        <v>12.30</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6">
         <v>2</v>
       </c>
-      <c r="D4" t="str">
-        <v>4.00</v>
-      </c>
-      <c r="E4" t="str">
-        <v>4.00</v>
-      </c>
-      <c r="F4" t="str">
+      <c r="B6" t="str">
+        <v>Cheesecake</v>
+      </c>
+      <c r="C6">
+        <v>2</v>
+      </c>
+      <c r="D6" t="str">
+        <v>5.00</v>
+      </c>
+      <c r="E6" t="str">
+        <v>5.00</v>
+      </c>
+      <c r="F6" t="str">
         <v>No</v>
       </c>
-      <c r="G4">
+      <c r="G6">
         <v>0</v>
       </c>
-      <c r="H4" t="str">
+      <c r="H6" t="str">
         <v>0.00</v>
       </c>
-      <c r="I4" t="str">
-        <v>8.00</v>
-      </c>
-      <c r="J4" t="str">
-        <v>3.00</v>
-      </c>
-      <c r="K4" t="str">
-        <v>5.00</v>
+      <c r="I6" t="str">
+        <v>10.00</v>
+      </c>
+      <c r="J6" t="str">
+        <v>4.40</v>
+      </c>
+      <c r="K6" t="str">
+        <v>5.60</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K6"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -671,10 +718,10 @@
         <v>Ana Maria</v>
       </c>
       <c r="B2" t="str">
-        <v>41.40</v>
+        <v>44.01</v>
       </c>
       <c r="C2">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>